<commit_message>
Update hierarchical binding and documentation
</commit_message>
<xml_diff>
--- a/specs/bindings/ADS_PSV_Binding.xlsx
+++ b/specs/bindings/ADS_PSV_Binding.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobuy\GitHub\UADA\UADC_PoC\specs\bindings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DFB6D1-0119-46C7-B0B3-07768891D814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADFEC31-D4C5-45DC-9212-06A7CF901C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7500" yWindow="5115" windowWidth="25860" windowHeight="11745" activeTab="1" xr2:uid="{8A31CEAE-9DE2-472F-9056-58C72E3AE39A}"/>
+    <workbookView xWindow="7980" yWindow="5865" windowWidth="20865" windowHeight="9660" activeTab="2" xr2:uid="{8A31CEAE-9DE2-472F-9056-58C72E3AE39A}"/>
   </bookViews>
   <sheets>
     <sheet name="EN16931_UBL_Invoice" sheetId="2" r:id="rId1"/>
     <sheet name="ADS_Invoices_Received" sheetId="1" r:id="rId2"/>
+    <sheet name="ADS_Invoices_Generated" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EN16931_UBL_Invoice!$A$1:$S$198</definedName>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2942" uniqueCount="1699">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3136" uniqueCount="1721">
   <si>
     <t>sequence</t>
   </si>
@@ -5121,6 +5122,72 @@
   </si>
   <si>
     <t>$.invoice.buyerAccountingReference[4]</t>
+  </si>
+  <si>
+    <t>auditdatastandards.O2C.july2015.pdf</t>
+  </si>
+  <si>
+    <t>Code for Tax2 type (for example, Sales, VAT). This field should agree with the Regulator_Code field in the Tax_Table_YYYYMMDD</t>
+  </si>
+  <si>
+    <t>Transaction monetary amount in local currency. Usually the amount seen on the original invoice document.</t>
+  </si>
+  <si>
+    <t>Grouping mechanism for related items in a batch or grouping of invoices, such as the invoice grouping found in certain ERP systems</t>
+  </si>
+  <si>
+    <t>Grouping_Code</t>
+  </si>
+  <si>
+    <t>Approved_Time</t>
+  </si>
+  <si>
+    <t>Date the entry was approved.</t>
+  </si>
+  <si>
+    <t>Approved_Date</t>
+  </si>
+  <si>
+    <t>User_ID (from User_Listing file) for person who approved customer master additions or changes.</t>
+  </si>
+  <si>
+    <t>Date the transaction was entered into the system. This is sometimes referred to as the creation date. This should be a system- generated date (rather than user-entered date), when possible. This date does not necessarily correspond with the date of the transaction itself.</t>
+  </si>
+  <si>
+    <t>The number of days from the invoice date the customer has to take advantage of discounted terms. Terms are represented as digits with no decimal places (for example, nnn).</t>
+  </si>
+  <si>
+    <t>The discount percentage the customer may take if an invoice is paid before a certain number of days. In the flat file, terms are represented as digits to one decimal place (for example, 10% would be represented as 10.0). In extensible business reporting language global ledger taxonomy framework (XBRL GL), the three fields Terms_Discount_Percentage, Terms_Discount_Days and Terms_Due_Days would be entered in the form "xx.x% dd Net dd," such as 2% 10 Net 30 for 2% discount if paid within 10 days, with the net due in 30 days.</t>
+  </si>
+  <si>
+    <t>Identifier of the customer from whom payment is expected or to whom unused credits have been applied. Must match a Customer_Account_ID in the Customer_Master_Listing_YYYYMMDD file.</t>
+  </si>
+  <si>
+    <t>Customer_Account_ID</t>
+  </si>
+  <si>
+    <t>Used to identify the business unit, region, branch, and so on at the level that financial statements are being audited. Must match a Business_Unit_Code in the Business_Unit_Listing file.</t>
+  </si>
+  <si>
+    <t>Sales order ID for invoiced items. Must match Sales_Order_ID in the Sales_Orders_YYYYMMDD_YYYYMMDD file. If no sales order, leave blank.</t>
+  </si>
+  <si>
+    <t>Sales_Order_ID</t>
+  </si>
+  <si>
+    <t>The date payment is due from the customer. Aging of a receivable is usually calculated based on this date.</t>
+  </si>
+  <si>
+    <t>Identification number for an internally generated invoice.</t>
+  </si>
+  <si>
+    <t>Unique identifier for each invoice. This ID may need to be created by concatenating fields (for example, document number, document type, and year) to uniquely identify each transaction. The same ID must be used for all tables with invoice data (Invoices_Generated_YYYYMMDD_YYYYM MDD, Open_Accounts_Receivable_YYYYMMDD, AR_Cash_Application_YYYYMMDD_YYYY MMDD, and AR_Adjustments_YYYYMMDD_YYYYMMD D).</t>
+  </si>
+  <si>
+    <t>Fiscal year in which the Invoice_Date occurs・E・EYYYY for delimited, CCYY-MM-DD fiscal year end (ISO 8601) for extensible business reporting language global ledger taxonomy framework (XBRL GL).</t>
+  </si>
+  <si>
+    <t>Fiscal period in which the Invoice_Date occurs. Examples include W1・E・EW53 for weekly periods, M1・E・EM12 for monthly periods, and Q1・E・EQ4 for quarterly periods.</t>
   </si>
 </sst>
 </file>
@@ -14846,7 +14913,7 @@
         <v>4</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>1621</v>
+        <v>1719</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>1618</v>
@@ -14872,7 +14939,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>1622</v>
+        <v>1720</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>1618</v>
@@ -15725,6 +15792,1021 @@
       </c>
       <c r="H42" t="s">
         <v>1698</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73A70007-E570-4E73-BE7F-C3B84723488C}">
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.375" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.25" customWidth="1"/>
+    <col min="5" max="5" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59.875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="31.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1612</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1613</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1614</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1615</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>1718</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>1717</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>1621</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>1622</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>1716</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C8" s="5">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>1714</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1625</v>
+      </c>
+      <c r="C9" s="5">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>1713</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H9" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C10" s="5">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>1711</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H10" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>1710</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C12" s="5">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>1709</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1632</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>1633</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C14" s="5">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>1635</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1636</v>
+      </c>
+      <c r="C15" s="5">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>1708</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C16" s="5">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1639</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>1640</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C17" s="5">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>1707</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1706</v>
+      </c>
+      <c r="C18" s="5">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1704</v>
+      </c>
+      <c r="C19" s="5">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1639</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>1646</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1647</v>
+      </c>
+      <c r="C20" s="5">
+        <v>2</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E20">
+        <v>100</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>1648</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C21" s="5">
+        <v>2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>1650</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C22" s="5">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1639</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>1652</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1703</v>
+      </c>
+      <c r="C23" s="5">
+        <v>2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E23">
+        <v>100</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>1702</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H23" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>1653</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H24" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E25">
+        <v>3</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>1654</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1655</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>1656</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E27">
+        <v>3</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>1658</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1659</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>1701</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C29" s="5">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>1662</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="5">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E30">
+        <v>25</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>1663</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1664</v>
+      </c>
+      <c r="C31" s="5">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E31">
+        <v>25</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>1700</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C32" s="5">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E32">
+        <v>25</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>1667</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E33">
+        <v>100</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>1668</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H33" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1669</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E34">
+        <v>100</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>1670</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1671</v>
+      </c>
+      <c r="C35" s="5">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E35">
+        <v>100</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>1672</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="5">
+        <v>2</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>1673</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H36" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1674</v>
+      </c>
+      <c r="C37" s="5">
+        <v>2</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>1675</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1676</v>
+      </c>
+      <c r="C38" s="5">
+        <v>2</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>1677</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C39" s="5">
+        <v>2</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E39">
+        <v>25</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H39" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C40" s="5">
+        <v>2</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E40">
+        <v>25</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C41" s="5">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E41">
+        <v>25</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1683</v>
+      </c>
+      <c r="C42" s="5">
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E42">
+        <v>25</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C43" s="5">
+        <v>2</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E43">
+        <v>25</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>1699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>